<commit_message>
Add governance docs, evaluation tooling, and review artifacts
Documents the safety posture that the code enforces: architecture and layer
boundaries, deployment modes, configuration, learning-data governance, LLM
review policy, retraining and promotion gates, and the human review guide.

Adds the offline scripts used to audit and evaluate the pipeline - retriever
and model evaluation, embedding audits, dry runs per phase, profiling, review
batch intake, and the sealed challenge-set guard. None of them run during
normal upload processing.

Includes the human-reviewed label artifacts and audit outputs that back the
evaluation claims, so the reported numbers are reproducible rather than
asserted.
</commit_message>
<xml_diff>
--- a/Product_Master.xlsx
+++ b/Product_Master.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://retailistancom-my.sharepoint.com/personal/muhammad_youshay_salesflo_com/Documents/Desktop/PromoPro - Al-Kabeer/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Internship\PromoStrater\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{401A57AA-BF36-4F7A-8840-C616EF3BB58A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3196FCA7-9D11-422D-A978-235B5836396C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F7983AE4-03E3-40A4-8DA8-AF9832FC6254}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{F7983AE4-03E3-40A4-8DA8-AF9832FC6254}"/>
   </bookViews>
   <sheets>
     <sheet name="Item" sheetId="1" r:id="rId1"/>
@@ -2382,20 +2382,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9F41802-782C-44DD-B8E4-78B7C6AE7945}">
   <dimension ref="A1:I238"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.88671875" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.88671875" customWidth="1"/>
-    <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="62.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.28515625" customWidth="1"/>
+    <col min="3" max="3" width="0.28515625" customWidth="1"/>
+    <col min="4" max="4" width="1.5703125" hidden="1" customWidth="1"/>
+    <col min="5" max="6" width="0.42578125" customWidth="1"/>
+    <col min="7" max="7" width="0.7109375" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="17.42578125" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="62.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2424,7 +2423,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -2454,7 +2453,7 @@
         <v>BEEF CUBES2 lb x 20 Pkts</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>16</v>
       </c>
@@ -2484,7 +2483,7 @@
         <v>BEEF TENDERLOIN/FILLET20 KGS</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>20</v>
       </c>
@@ -2514,7 +2513,7 @@
         <v>BEEF TOPSIDE ALK20 KGS</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>22</v>
       </c>
@@ -2544,7 +2543,7 @@
         <v>VEAL LEGS 3.6Asstd. Wt.</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
@@ -2574,7 +2573,7 @@
         <v>AK PRO BEEF BURGER 241.392 kg x 6 Pkts</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>32</v>
       </c>
@@ -2604,7 +2603,7 @@
         <v>CHAR.JUMBO BEEF BURGERS BULK(100G)6*1 KG1KG X 6</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>36</v>
       </c>
@@ -2634,7 +2633,7 @@
         <v>4 BEEF BURGERS200 Gms x 30 Pkt</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
@@ -2664,7 +2663,7 @@
         <v>24 BEEF BURGERS1.2 Kgs x 8 Pkts</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>42</v>
       </c>
@@ -2694,7 +2693,7 @@
         <v>BEEF BURGERS BULK2 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>45</v>
       </c>
@@ -2724,7 +2723,7 @@
         <v>TAYEBAT BEEF BURGERS ONION BULK1 Kgs x 9 Pkts</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>48</v>
       </c>
@@ -2754,7 +2753,7 @@
         <v>BEEF BURGERS 56 g.840 g. x 9</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>51</v>
       </c>
@@ -2784,7 +2783,7 @@
         <v>BEEF KIBBEH 400400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>55</v>
       </c>
@@ -2814,7 +2813,7 @@
         <v>CHICKEN BIRYANI 400400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>59</v>
       </c>
@@ -2844,7 +2843,7 @@
         <v>CHICKEN TIKKA MAKHANI &amp; PILAU RICE450 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>62</v>
       </c>
@@ -2874,7 +2873,7 @@
         <v>CHICKEN FRIES12 PKTS X 400 GRM</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>66</v>
       </c>
@@ -2904,7 +2903,7 @@
         <v>CHICKEN FRIES BULK1 kg x 5 Pkts</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>69</v>
       </c>
@@ -2934,7 +2933,7 @@
         <v>CHICKEN STICKS BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>73</v>
       </c>
@@ -2964,7 +2963,7 @@
         <v>CHICKEN STICK BULK HOT &amp; SPICY1 kg x 5 Pkts</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>75</v>
       </c>
@@ -2994,7 +2993,7 @@
         <v>MOZZERELLA CHEESE STICKS250 GMS X24 PKTS</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>79</v>
       </c>
@@ -3024,7 +3023,7 @@
         <v>MOZZARELLA CHEESE STICKS1000G X 5 Pkts</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
@@ -3054,7 +3053,7 @@
         <v>12 CHEESE SAMOSAS240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>86</v>
       </c>
@@ -3084,7 +3083,7 @@
         <v>CHEESE SAMOSAS BULK1.2 Kgs x 4 Pkts</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>89</v>
       </c>
@@ -3114,7 +3113,7 @@
         <v>A.K PRO CHEESE SAMOSA4 X 1.2 KGS</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>92</v>
       </c>
@@ -3144,7 +3143,7 @@
         <v>KIRI CHEESE SAMOSA20 X 240 GMS</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>95</v>
       </c>
@@ -3174,7 +3173,7 @@
         <v>Kiri Cheese &amp; Jalapeño Samosas 240 g. X 2020 X 240 GMS</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>97</v>
       </c>
@@ -3204,7 +3203,7 @@
         <v>Kiri Cheese &amp; Zaatar Samosas 240 g. X 2020 X 240 GMS</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>99</v>
       </c>
@@ -3234,7 +3233,7 @@
         <v>8 CHEESE SPRING ROLLS240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>102</v>
       </c>
@@ -3264,7 +3263,7 @@
         <v>BEEF FRANKS454 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>106</v>
       </c>
@@ -3294,7 +3293,7 @@
         <v>BREADED FISH FILLET330 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>111</v>
       </c>
@@ -3324,7 +3323,7 @@
         <v>BREADED FISH FILLET BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>113</v>
       </c>
@@ -3354,7 +3353,7 @@
         <v>JUMBO HOTDOGS400 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>116</v>
       </c>
@@ -3384,7 +3383,7 @@
         <v>FISH FINGERS 300300 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>119</v>
       </c>
@@ -3414,7 +3413,7 @@
         <v>FISH STICKS BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
         <v>121</v>
       </c>
@@ -3444,7 +3443,7 @@
         <v>ZING FISH FILLETS MILD SPICY750 g. x 8</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
         <v>125</v>
       </c>
@@ -3474,7 +3473,7 @@
         <v>ARABIC KOFTA300 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>127</v>
       </c>
@@ -3504,7 +3503,7 @@
         <v>AK PRO CHICKEN BURGER 241.392 kg x 6 Pkts</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>129</v>
       </c>
@@ -3534,7 +3533,7 @@
         <v>8 BREADED CHICKEN BURGERS400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>131</v>
       </c>
@@ -3564,7 +3563,7 @@
         <v>BREADED CHICKEN BURGERS 50GM CAT1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>133</v>
       </c>
@@ -3594,7 +3593,7 @@
         <v>Breaded Chicken Burger Bag (56 g.)840 g. x 9</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>135</v>
       </c>
@@ -3624,7 +3623,7 @@
         <v>AK PRO Breaded Chicken Burger Bag 840 g. x 8840 gm x 8</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>138</v>
       </c>
@@ -3654,7 +3653,7 @@
         <v>8 BREADED CHICKEN BURGER HOT &amp; SPICY400 gm x 12 Pkts</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>141</v>
       </c>
@@ -3684,7 +3683,7 @@
         <v>TAYEBAT BREADED CHICKEN BURGERS BULK900 Gms x 9 Pkts</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>144</v>
       </c>
@@ -3714,7 +3713,7 @@
         <v>TAYEBAT BREADED CHICKEN BURGERS 840 g. x 8 Pkts840 g. x 8 Pkts</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>147</v>
       </c>
@@ -3744,7 +3743,7 @@
         <v>BREADED CHICKEN FILLETS450 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>149</v>
       </c>
@@ -3774,7 +3773,7 @@
         <v>AK PRO Breaded Chicken Fillets10X1000g</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>152</v>
       </c>
@@ -3804,7 +3803,7 @@
         <v>BREADED CHICKEN FILLETS HOT N SPICY330 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>154</v>
       </c>
@@ -3834,7 +3833,7 @@
         <v>BREADED CHICKEN FILLETS HOT N SPICY BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>157</v>
       </c>
@@ -3864,7 +3863,7 @@
         <v>BREADED CHICKEN FILLET SPICY 750 GMS750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>160</v>
       </c>
@@ -3894,7 +3893,7 @@
         <v>BREADED CHICKEN FILLET NON-SPICY 750 GMS750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>162</v>
       </c>
@@ -3924,7 +3923,7 @@
         <v>Breaded Chicken Fillets Non Spicy +33% Free(750 g. + 250 g.) x 8</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
         <v>166</v>
       </c>
@@ -3954,7 +3953,7 @@
         <v>BREADED CHICKEN FILLETS BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
         <v>168</v>
       </c>
@@ -3984,7 +3983,7 @@
         <v>BEEF COCKTAIL SAUSAGES400 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
         <v>170</v>
       </c>
@@ -4014,7 +4013,7 @@
         <v>TAYEBAT BEEF MEAT BALLS 1 kg x 10 Pkts1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
         <v>174</v>
       </c>
@@ -4044,7 +4043,7 @@
         <v>8 BEEF SEEKH KEBAB320 Gms x 24 Pkts</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
         <v>178</v>
       </c>
@@ -4074,7 +4073,7 @@
         <v>TAYEBAT CHICKEN BURGER1 Kgs x 9 Pkts</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
         <v>180</v>
       </c>
@@ -4104,7 +4103,7 @@
         <v>TAYEBAT CHICKEN BURGERS 1 kg x 10 Pkts1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
         <v>182</v>
       </c>
@@ -4134,7 +4133,7 @@
         <v>BBQ CHICKEN WINGS 400400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
         <v>185</v>
       </c>
@@ -4164,7 +4163,7 @@
         <v>CHICKEN  N CHEESE NUGGETS400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
         <v>188</v>
       </c>
@@ -4194,7 +4193,7 @@
         <v>CHICKEN &amp; CHEESE STICKS HOT &amp; SPICY250 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
         <v>191</v>
       </c>
@@ -4224,7 +4223,7 @@
         <v>CHICKEN ‘N’ CHEESE RINGS 300300 gms x 12 pkts</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
         <v>194</v>
       </c>
@@ -4254,7 +4253,7 @@
         <v>CHICKEN &amp; CHEESE STICKS250 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
         <v>197</v>
       </c>
@@ -4284,7 +4283,7 @@
         <v>CHICKEN &amp; CHEESE STICKS BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
         <v>199</v>
       </c>
@@ -4314,7 +4313,7 @@
         <v>CHICKEN &amp; CHEESE STICKS SPICY BULK1 kg x 5 Pkts</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
         <v>201</v>
       </c>
@@ -4344,7 +4343,7 @@
         <v>CHICKEN &amp; CHEESE STICKS TWIN PROMO PACK250GMSx2PKTx10</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
         <v>205</v>
       </c>
@@ -4374,7 +4373,7 @@
         <v>CHICKEN KOFTA 300300 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
         <v>207</v>
       </c>
@@ -4404,7 +4403,7 @@
         <v>CHICKEN BURGERS 56 g840 g. x 9</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
         <v>209</v>
       </c>
@@ -4434,7 +4433,7 @@
         <v>CHICKEN MINCE 400400 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
         <v>213</v>
       </c>
@@ -4464,7 +4463,7 @@
         <v>CHICKEN MINCE (15% FREE )400+60 G X 20 Pkts</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
         <v>217</v>
       </c>
@@ -4494,7 +4493,7 @@
         <v>8 CHICKEN SEEKH KEBAB320 Gms x 24 Pkts</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
         <v>219</v>
       </c>
@@ -4524,7 +4523,7 @@
         <v>CHICKEN SEEKH KEBAB BULK1 kg x 5</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="2" t="s">
         <v>222</v>
       </c>
@@ -4554,7 +4553,7 @@
         <v>TAYEBAT BREADED CHICKEN FILLETS NON SPICY 1 kg x 10 Pkts1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
         <v>224</v>
       </c>
@@ -4584,7 +4583,7 @@
         <v>JUMBO CHICKEN NUGGETS1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
         <v>226</v>
       </c>
@@ -4614,7 +4613,7 @@
         <v>JUMBO CHICKEN STICKS (BULK)1 kg x 5 Pkts</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
         <v>228</v>
       </c>
@@ -4644,7 +4643,7 @@
         <v>CHICKEN KIBBEH 400400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
         <v>230</v>
       </c>
@@ -4674,7 +4673,7 @@
         <v>4 CHICKEN BURGERS200 Gms x 30 Pkts</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
         <v>233</v>
       </c>
@@ -4704,7 +4703,7 @@
         <v>CHARGRILLED JUMBO CHICKEN BURGERS1  kgs x 6 pkts</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
         <v>236</v>
       </c>
@@ -4734,7 +4733,7 @@
         <v>24 CHICKEN BURGERS1.2 Kgs x 8 Pkts</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
         <v>238</v>
       </c>
@@ -4764,7 +4763,7 @@
         <v>24 CHICKEN BURGERS BULK2 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
         <v>240</v>
       </c>
@@ -4794,7 +4793,7 @@
         <v>24 CHICKEN BURGERS (4PCS FREE)1.4 kg x 8</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
         <v>243</v>
       </c>
@@ -4824,7 +4823,7 @@
         <v>AK PRO Chicken Burger 50 g. 1 kg x 101 kg x 10</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
         <v>246</v>
       </c>
@@ -4854,7 +4853,7 @@
         <v>8 CHICKEN BURGERS400 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
         <v>248</v>
       </c>
@@ -4884,7 +4883,7 @@
         <v>JUMBO BREADED CHICKEN BURGER 100G BULK1000 GM X 6 PKTS</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
         <v>251</v>
       </c>
@@ -4914,7 +4913,7 @@
         <v>CHICKEN MEAT BALLS300 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
         <v>253</v>
       </c>
@@ -4944,7 +4943,7 @@
         <v>CHICKEN MEAT BALLS BULK1 Kgs x 6 Pkts</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
         <v>256</v>
       </c>
@@ -4974,7 +4973,7 @@
         <v>CHICKEN MEAT BALLS CATERING PACK 1 kg x 5 pkts1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
         <v>258</v>
       </c>
@@ -5004,7 +5003,7 @@
         <v>TENDER CHICKEN BREAST1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
         <v>261</v>
       </c>
@@ -5034,7 +5033,7 @@
         <v>TENDER CHICKEN BREAST SPICY FLAVOURED2 KG X 6 PKT</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
         <v>264</v>
       </c>
@@ -5064,7 +5063,7 @@
         <v>CHICKEN NUGGETS270 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
         <v>267</v>
       </c>
@@ -5094,7 +5093,7 @@
         <v>CHICKEN NUGGETS (400G)400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
         <v>269</v>
       </c>
@@ -5124,7 +5123,7 @@
         <v>CHICKEN NUGGETS BULK 1x51 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="2" t="s">
         <v>271</v>
       </c>
@@ -5154,7 +5153,7 @@
         <v>CHICKEN NUGGETS 750 GMS750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="2" t="s">
         <v>273</v>
       </c>
@@ -5184,7 +5183,7 @@
         <v>Chicken Nuggets +33% Free(750 g. + 250 g.) x 8</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="2" t="s">
         <v>275</v>
       </c>
@@ -5214,7 +5213,7 @@
         <v>AK PRO CHICKEN NUGGETS BULK10 X 1000 GMS</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="2" t="s">
         <v>278</v>
       </c>
@@ -5244,7 +5243,7 @@
         <v>Chicken Nuggets + Free Chicken Samosa Combo Pack(750 g. + 240 g.) x 6</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="2" t="s">
         <v>282</v>
       </c>
@@ -5274,7 +5273,7 @@
         <v>CHICKEN NUGGETS HOT &amp; SPICY BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="2" t="s">
         <v>284</v>
       </c>
@@ -5304,7 +5303,7 @@
         <v>Chicken Nuggets HOT n SPICY750 g. x 8</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="2" t="s">
         <v>286</v>
       </c>
@@ -5334,7 +5333,7 @@
         <v>KRAZEE CHICKEN NUGGETS 400400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="2" t="s">
         <v>288</v>
       </c>
@@ -5364,7 +5363,7 @@
         <v>KRAZEE CHICKEN NUGGETS SPICY 750 GRM750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="2" t="s">
         <v>290</v>
       </c>
@@ -5394,7 +5393,7 @@
         <v>Krazee Chicken Nuggets +33% Free(750 g. + 250 g.) x 8</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="2" t="s">
         <v>292</v>
       </c>
@@ -5424,7 +5423,7 @@
         <v>KRAZEE CHICKEN NUGGETS TWIN PROMO PACK400 Gmsx2Pktx6</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="2" t="s">
         <v>295</v>
       </c>
@@ -5454,7 +5453,7 @@
         <v>KRAZEE CHICKEN NUGGETS +25% FREE500Gms X 12Ctn</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="2" t="s">
         <v>298</v>
       </c>
@@ -5484,7 +5483,7 @@
         <v>AK PRO Chicken Nuggets 1 kg x 1010 X 1000 GMS</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="2" t="s">
         <v>300</v>
       </c>
@@ -5514,7 +5513,7 @@
         <v>Tempura Chicken Nuggets Non Spicy750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="2" t="s">
         <v>302</v>
       </c>
@@ -5544,7 +5543,7 @@
         <v>TAYEBAT CHICKEN NUGGETS 1 kg x 10 Pkts1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="2" t="s">
         <v>304</v>
       </c>
@@ -5574,7 +5573,7 @@
         <v>CHICKEN POP-CORN400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="2" t="s">
         <v>307</v>
       </c>
@@ -5604,7 +5603,7 @@
         <v>CHICKEN POP-CORN 750 GMS750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="2" t="s">
         <v>309</v>
       </c>
@@ -5634,7 +5633,7 @@
         <v>AK PRO Plain Chicken Strips 30 g. 1 kg x 101 kg x 10</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>312</v>
       </c>
@@ -5664,7 +5663,7 @@
         <v>12 CHICKEN SAMOSAS240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" s="2" t="s">
         <v>314</v>
       </c>
@@ -5694,7 +5693,7 @@
         <v>CHICKEN SAMOSAS BULK1.2 Kgs x 4 Pkts</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" s="2" t="s">
         <v>316</v>
       </c>
@@ -5724,7 +5723,7 @@
         <v>CHICKEN SAMOSAS TWIN PROMO PACK480 Gms x 10 Pkts</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" s="2" t="s">
         <v>319</v>
       </c>
@@ -5754,7 +5753,7 @@
         <v>AK PRO CHICKEN SAMOSA4 X 1.2 KGS</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" s="2" t="s">
         <v>321</v>
       </c>
@@ -5784,7 +5783,7 @@
         <v>SHISH KEBAB600 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" s="2" t="s">
         <v>324</v>
       </c>
@@ -5814,7 +5813,7 @@
         <v>8 CHICKEN SPRING ROLLS280 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" s="2" t="s">
         <v>327</v>
       </c>
@@ -5844,7 +5843,7 @@
         <v>CHICKEN SPRING ROLL BULK (5*1120G)1.12 kg x 5 pkts</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
         <v>330</v>
       </c>
@@ -5874,7 +5873,7 @@
         <v>8 CHICKEN SPRING ROLLS TWIN PROMO PACK560 Gms x 10 Pkts</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
         <v>333</v>
       </c>
@@ -5904,7 +5903,7 @@
         <v>SHISH TAWOOK240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
         <v>336</v>
       </c>
@@ -5934,7 +5933,7 @@
         <v>SHISH TAWOOK BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
         <v>338</v>
       </c>
@@ -5964,7 +5963,7 @@
         <v>TAYEBAT BREADED CHICKEN STRIPS NON SPICY 1 kg x 10 Pkts1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
         <v>340</v>
       </c>
@@ -5994,7 +5993,7 @@
         <v>TENDER CHICKEN BREAST TRAY PACK450 GMS X 10 PKTS</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
         <v>343</v>
       </c>
@@ -6024,7 +6023,7 @@
         <v>TURKISH CHICKEN KEBAB360gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
         <v>346</v>
       </c>
@@ -6054,7 +6053,7 @@
         <v>TANDOORI CHICKEN TIKKA240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
         <v>348</v>
       </c>
@@ -6084,7 +6083,7 @@
         <v>TANDOORI CHICKEN TIKKA BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
         <v>350</v>
       </c>
@@ -6114,7 +6113,7 @@
         <v>TANDOORI CHICKEN NUGGETS 270270 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
         <v>352</v>
       </c>
@@ -6144,7 +6143,7 @@
         <v>ZING CHICKEN FILLETS 465465 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
         <v>355</v>
       </c>
@@ -6174,7 +6173,7 @@
         <v>ZING CHICKEN FILLETS BULK (5*1 KG)1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
         <v>357</v>
       </c>
@@ -6204,7 +6203,7 @@
         <v>ZING CHICKEN FILLET BULK 5-OUNCE5 PKTS X 1000 GRM</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
         <v>360</v>
       </c>
@@ -6234,7 +6233,7 @@
         <v>Zing Chicken Fillets Spicy + Free Chicken Nuggets1kg+750 g. x 3</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
         <v>363</v>
       </c>
@@ -6264,7 +6263,7 @@
         <v>Butter Chicken Zing Fillets 700 g. x 8700 g. x 8</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
         <v>366</v>
       </c>
@@ -6294,7 +6293,7 @@
         <v>Zing Chicken Fillets Spicy + Free Chicken Fries Bulk1+1 kg x 3</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
         <v>369</v>
       </c>
@@ -6324,7 +6323,7 @@
         <v>ZING CHICKEN FILLETS SPICY 750 GRM750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
         <v>371</v>
       </c>
@@ -6354,7 +6353,7 @@
         <v>Zing Chicken Fillets 5-Ounce750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
         <v>373</v>
       </c>
@@ -6384,7 +6383,7 @@
         <v>Zing Chicken Fillets Tamiya750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
         <v>375</v>
       </c>
@@ -6414,7 +6413,7 @@
         <v>ZING CHICKEN FILLET NON-SPICY8 X 750 GMS</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
         <v>378</v>
       </c>
@@ -6444,7 +6443,7 @@
         <v>ZING CHICKEN LOLLIPOP 420420 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
         <v>382</v>
       </c>
@@ -6474,7 +6473,7 @@
         <v>ZING CHICKEN LOLLIPOP BULK (5*1KG)1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
         <v>384</v>
       </c>
@@ -6504,7 +6503,7 @@
         <v>ZING CHICKEN NUGGETS REGULAR270 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
         <v>386</v>
       </c>
@@ -6534,7 +6533,7 @@
         <v>ZING CHICKEN NUGGET NON-SPICY8 X 750 GMS</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" s="2" t="s">
         <v>388</v>
       </c>
@@ -6564,7 +6563,7 @@
         <v>ZING CHICKEN STRIPS320 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" s="2" t="s">
         <v>391</v>
       </c>
@@ -6594,7 +6593,7 @@
         <v>Zing Strips Non Spicy + Free Chicken Nuggets Combo Pack(750 g.+750 g.) x 4</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" s="2" t="s">
         <v>395</v>
       </c>
@@ -6624,7 +6623,7 @@
         <v>ZING CHICKEN STRIPS SPICY 750 GRM750 GMS X 8 PKT</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" s="2" t="s">
         <v>397</v>
       </c>
@@ -6654,7 +6653,7 @@
         <v>ZING CHICKEN STRIPS NON-SPICY8 X 750 GMS</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" s="2" t="s">
         <v>399</v>
       </c>
@@ -6684,7 +6683,7 @@
         <v>AK PRO Zing Chicken Strips Non Spicy 1 kg x 101kg X 10pkts</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" s="2" t="s">
         <v>402</v>
       </c>
@@ -6714,7 +6713,7 @@
         <v>ZING CHICKEN STRIPS -SMOKEY BUFFALO700 GM X 8 PKT</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" s="2" t="s">
         <v>405</v>
       </c>
@@ -6744,7 +6743,7 @@
         <v>ZING CHICKEN STRIPS SRIRACHA700 GM X 8 PKT</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" s="2" t="s">
         <v>407</v>
       </c>
@@ -6774,7 +6773,7 @@
         <v>LAMB KIBBEH400 Gms x 12 Pkts</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" s="2" t="s">
         <v>409</v>
       </c>
@@ -6804,7 +6803,7 @@
         <v>LAMB KIBBEH BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" s="2" t="s">
         <v>411</v>
       </c>
@@ -6834,7 +6833,7 @@
         <v>MEAT BALLS300 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" s="2" t="s">
         <v>412</v>
       </c>
@@ -6864,7 +6863,7 @@
         <v>MEAT BALLS BULK1 kg x 6  Pkts</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" s="2" t="s">
         <v>415</v>
       </c>
@@ -6894,7 +6893,7 @@
         <v>AK PRO Beef Meat Balls 1 kg x 101 kg x 10</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" s="2" t="s">
         <v>417</v>
       </c>
@@ -6924,7 +6923,7 @@
         <v>12 MUTTON SAMOSAS240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" s="2" t="s">
         <v>419</v>
       </c>
@@ -6954,7 +6953,7 @@
         <v>MUTTON SAMOSAS BULK1.2 Kgs x 4 Pkts</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" s="2" t="s">
         <v>421</v>
       </c>
@@ -6984,7 +6983,7 @@
         <v>chocolate Samosas 240 g x 20240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" s="2" t="s">
         <v>423</v>
       </c>
@@ -7014,7 +7013,7 @@
         <v>BREADED SHRIMPS 250250 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" s="2" t="s">
         <v>426</v>
       </c>
@@ -7044,7 +7043,7 @@
         <v>BREADED SHRIMPS BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" s="2" t="s">
         <v>428</v>
       </c>
@@ -7074,7 +7073,7 @@
         <v>JUMBO PRAWNS1 lb x 10 Pkts</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" s="2" t="s">
         <v>431</v>
       </c>
@@ -7104,7 +7103,7 @@
         <v>PRAWNS LARGE 400400 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" s="2" t="s">
         <v>433</v>
       </c>
@@ -7134,7 +7133,7 @@
         <v>PRAWNS MEDIUM 400400 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" s="2" t="s">
         <v>435</v>
       </c>
@@ -7164,7 +7163,7 @@
         <v>AK PRO JUMBO PRAWN CRISPIES10 X 1 KGS</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" s="2" t="s">
         <v>438</v>
       </c>
@@ -7194,7 +7193,7 @@
         <v>PRAWNS REGULAR400 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" s="2" t="s">
         <v>440</v>
       </c>
@@ -7224,7 +7223,7 @@
         <v>TABARRUK COOKING SHRIMPS BULK1 Kgs x 10 Pkts</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" s="2" t="s">
         <v>443</v>
       </c>
@@ -7254,7 +7253,7 @@
         <v>TABARRUK COOKING SHRIMPS FAMILY PACK500 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" s="2" t="s">
         <v>446</v>
       </c>
@@ -7284,7 +7283,7 @@
         <v>PRAWNS EXTRA LARGE400 Gms x 10 Pkts</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" s="2" t="s">
         <v>449</v>
       </c>
@@ -7314,7 +7313,7 @@
         <v>TURKISH BEEF KEBABS 360360GM X 20 PKT</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" s="2" t="s">
         <v>452</v>
       </c>
@@ -7344,7 +7343,7 @@
         <v>FELAFEL360 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" s="2" t="s">
         <v>455</v>
       </c>
@@ -7374,7 +7373,7 @@
         <v>FELAFEL BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" s="2" t="s">
         <v>457</v>
       </c>
@@ -7404,7 +7403,7 @@
         <v>FELAFEL GREEN BULK1 Kgs x 5 Pkts</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" s="2" t="s">
         <v>459</v>
       </c>
@@ -7434,7 +7433,7 @@
         <v>JALAPENO &amp; CHEESE STICKS 250250 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" s="2" t="s">
         <v>461</v>
       </c>
@@ -7464,7 +7463,7 @@
         <v>FROZEN PUNJABI SAMOSA900GM X 10PKT</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
         <v>464</v>
       </c>
@@ -7494,7 +7493,7 @@
         <v>12 VEGETABLE SAMOSAS240 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" s="2" t="s">
         <v>466</v>
       </c>
@@ -7524,7 +7523,7 @@
         <v>VEGETABLE SAMOSAS BULK1.2 Kgs x 4 Pkts</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" s="2" t="s">
         <v>468</v>
       </c>
@@ -7554,7 +7553,7 @@
         <v>VEGETABLE SAMOSA TWIN PROMO PACK480 Gms x 10 Pkts</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" s="2" t="s">
         <v>470</v>
       </c>
@@ -7584,7 +7583,7 @@
         <v>AK PRO VEGETABLE SAMOSA1.2 Kgs x 4 Pkts</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" s="2" t="s">
         <v>472</v>
       </c>
@@ -7614,7 +7613,7 @@
         <v>STUFFED FELAFEL750 g. x 8</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" s="2" t="s">
         <v>474</v>
       </c>
@@ -7644,7 +7643,7 @@
         <v>8 VEGETABLE SPRING ROLLS280 Gms x 20 Pkts</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" s="2" t="s">
         <v>476</v>
       </c>
@@ -7674,7 +7673,7 @@
         <v>VEGETABLE SPRING ROLLS BULK (5*1120G)1.12 kg x 5 pkts</v>
       </c>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" s="2" t="s">
         <v>478</v>
       </c>
@@ -7704,7 +7703,7 @@
         <v>8 VEGETABLE SPRING ROLLS TWIN PROMO PACK560 Gms x 10 Pkts</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" s="2" t="s">
         <v>480</v>
       </c>
@@ -7734,7 +7733,7 @@
         <v>Zing Chicken Fillets Non Spicy + Free Chicken Fillets Spicy750+750 g. x 4</v>
       </c>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A179" s="2" t="s">
         <v>483</v>
       </c>
@@ -7764,7 +7763,7 @@
         <v>Zing Shrimps750 gm x 8 Pkts</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" s="2" t="s">
         <v>486</v>
       </c>
@@ -7794,7 +7793,7 @@
         <v>CREAM DORI FISH FILLETSAsstd. Wt.</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" s="2" t="s">
         <v>489</v>
       </c>
@@ -7824,7 +7823,7 @@
         <v>WHITE FISH FILLET 1KG1kg X 10 Pkts</v>
       </c>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" s="2" t="s">
         <v>492</v>
       </c>
@@ -7854,7 +7853,7 @@
         <v>AK PRO FISH FILLET2 KGS X 5</v>
       </c>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" s="2" t="s">
         <v>495</v>
       </c>
@@ -7884,7 +7883,7 @@
         <v>TABARRUK SUTCHI FISH FILLET2kg X 5pkts</v>
       </c>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" s="2" t="s">
         <v>498</v>
       </c>
@@ -7914,7 +7913,7 @@
         <v>BONELESS VEAL LOCAL20 X 2 LB</v>
       </c>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" s="2" t="s">
         <v>502</v>
       </c>
@@ -7944,7 +7943,7 @@
         <v>FROZEN QUAIL600 gm x 18 Pkts</v>
       </c>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" s="2" t="s">
         <v>505</v>
       </c>
@@ -7974,7 +7973,7 @@
         <v>MUTTON CUBES2 lbs x 20 Pkts</v>
       </c>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" s="2" t="s">
         <v>508</v>
       </c>
@@ -8004,7 +8003,7 @@
         <v>MUTTON RIB CHOPS1 lb x 40 Pkts</v>
       </c>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" s="2" t="s">
         <v>511</v>
       </c>
@@ -8034,7 +8033,7 @@
         <v>FISH MILK1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" s="2" t="s">
         <v>514</v>
       </c>
@@ -8064,7 +8063,7 @@
         <v>PARATHA PLAIN PROMO  400gmsx3 Pktsx8400 gm x 3 Pkts x 8</v>
       </c>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" s="2" t="s">
         <v>518</v>
       </c>
@@ -8094,7 +8093,7 @@
         <v>BLACKBERRIES 350GM350 gms x 20</v>
       </c>
     </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" s="2" t="s">
         <v>523</v>
       </c>
@@ -8124,7 +8123,7 @@
         <v>BLUEBERRY400 gms x 20</v>
       </c>
     </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" s="2" t="s">
         <v>526</v>
       </c>
@@ -8154,7 +8153,7 @@
         <v>BLUEBERRIES 350GM350 gms x 20</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" s="2" t="s">
         <v>528</v>
       </c>
@@ -8184,7 +8183,7 @@
         <v>BONELESS CHICKEN BREAST 102 kg x 5 Pkts</v>
       </c>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A194" s="2" t="s">
         <v>531</v>
       </c>
@@ -8214,7 +8213,7 @@
         <v>8 CORN ON THE COB628 G X 12</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A195" s="2" t="s">
         <v>536</v>
       </c>
@@ -8244,7 +8243,7 @@
         <v>CORN ON THE COB1 kg x 12 Pkts</v>
       </c>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A196" s="2" t="s">
         <v>539</v>
       </c>
@@ -8274,7 +8273,7 @@
         <v>AK PRO French Fries 2.5 kg x 4 (6x6 MM)2.5 kg x 4</v>
       </c>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A197" s="2" t="s">
         <v>543</v>
       </c>
@@ -8304,7 +8303,7 @@
         <v>AK PRO French Fries Salted &amp; Coated 2.5 kg x 4 (6x6 MM)2.5 Kgs x 6</v>
       </c>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A198" s="2" t="s">
         <v>546</v>
       </c>
@@ -8334,7 +8333,7 @@
         <v>FRENCH FRIES 2.5x42.5 kg x 4 Pkts</v>
       </c>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A199" s="2" t="s">
         <v>550</v>
       </c>
@@ -8364,7 +8363,7 @@
         <v>AK PRO FRENCH FRIES BULK2.5 kg x 4 Pkts</v>
       </c>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A200" s="2" t="s">
         <v>552</v>
       </c>
@@ -8394,7 +8393,7 @@
         <v>Chicken Frank 340 G  x 24340 gm x 24 Pkts</v>
       </c>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A201" s="2" t="s">
         <v>555</v>
       </c>
@@ -8424,7 +8423,7 @@
         <v>FRENCH FRIES 11 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A202" s="2" t="s">
         <v>557</v>
       </c>
@@ -8454,7 +8453,7 @@
         <v>Thin Cut French Fries 1 kg x 10 pkts1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A203" s="2" t="s">
         <v>559</v>
       </c>
@@ -8484,7 +8483,7 @@
         <v>CHICKEN JUMBO HOT DOGS400 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A204" s="2" t="s">
         <v>562</v>
       </c>
@@ -8514,7 +8513,7 @@
         <v>Chicken jumbo Hot Dogs 400 g x  24400 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A205" s="2" t="s">
         <v>564</v>
       </c>
@@ -8544,7 +8543,7 @@
         <v>HASH BROWNS2.5 kg x 4 Pkts</v>
       </c>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A206" s="2" t="s">
         <v>567</v>
       </c>
@@ -8574,7 +8573,7 @@
         <v>HASH BROWN10  X 1 KG</v>
       </c>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>570</v>
       </c>
@@ -8604,7 +8603,7 @@
         <v>Chicken Cocktail  Frank 300 G  x 24300 gm x 24 Pkts</v>
       </c>
     </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>573</v>
       </c>
@@ -8634,7 +8633,7 @@
         <v>MIX BERRIES 400x20400GMx 20</v>
       </c>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>576</v>
       </c>
@@ -8664,7 +8663,7 @@
         <v>Mix Berries 350 g. x 20350x20</v>
       </c>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>579</v>
       </c>
@@ -8694,7 +8693,7 @@
         <v>MANGO PULP NEW1 kgs x 16 Pkts</v>
       </c>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>582</v>
       </c>
@@ -8724,7 +8723,7 @@
         <v>MANGO SLICES1 Kgs x 10 Pkts</v>
       </c>
     </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>584</v>
       </c>
@@ -8754,7 +8753,7 @@
         <v>PANEER CUBES200 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>587</v>
       </c>
@@ -8784,7 +8783,7 @@
         <v>PANEER CUBES 500500 gm x 10 Pkts</v>
       </c>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>590</v>
       </c>
@@ -8814,7 +8813,7 @@
         <v>POTATO BITES1 Kgs x 10 Pkts</v>
       </c>
     </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>592</v>
       </c>
@@ -8844,7 +8843,7 @@
         <v>Chocolate Paratha 270 g. x 24270 Gms x 24 Pkts</v>
       </c>
     </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A216" s="2" t="s">
         <v>596</v>
       </c>
@@ -8874,7 +8873,7 @@
         <v>MALABAR PARATHA400G. X 24Pkts.</v>
       </c>
     </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>599</v>
       </c>
@@ -8904,7 +8903,7 @@
         <v>PLAIN PARATHA400 gm x 24 Pkts</v>
       </c>
     </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>602</v>
       </c>
@@ -8934,7 +8933,7 @@
         <v>PLAIN PARATHA PROMO1200 gm x 8 Pkts</v>
       </c>
     </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>605</v>
       </c>
@@ -8964,7 +8963,7 @@
         <v>PARATHA ROLL WHEAT400 gm x 24 Pkts</v>
       </c>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>607</v>
       </c>
@@ -8994,7 +8993,7 @@
         <v>Plain Paratha + Free Wheat Paratha Promo 400+400 g. x 12400+400G X 12</v>
       </c>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
         <v>610</v>
       </c>
@@ -9024,7 +9023,7 @@
         <v>PUNJABI SAMOSA450 GMS X 10 PKTS</v>
       </c>
     </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
         <v>612</v>
       </c>
@@ -9054,7 +9053,7 @@
         <v>TAY. PARATHA PLAIN400 gm x 24 Pkts</v>
       </c>
     </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>614</v>
       </c>
@@ -9084,7 +9083,7 @@
         <v>STRAWBERRIES900 gm x 10 Pkts</v>
       </c>
     </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A224" s="2" t="s">
         <v>617</v>
       </c>
@@ -9114,7 +9113,7 @@
         <v>AK PRO Strawberries 1 kg x 81kg x 8</v>
       </c>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
         <v>620</v>
       </c>
@@ -9144,7 +9143,7 @@
         <v>SWEET CORN 400400 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
         <v>622</v>
       </c>
@@ -9174,7 +9173,7 @@
         <v>SWEET CORN BULK1 kg x 10 Pkts</v>
       </c>
     </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
         <v>624</v>
       </c>
@@ -9204,7 +9203,7 @@
         <v>SEASONED WEDGES750 gm x 12 Pkts</v>
       </c>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A228" s="2" t="s">
         <v>627</v>
       </c>
@@ -9234,7 +9233,7 @@
         <v>TORTILLA WRAPS HOT  N  SPICY 10.5"875 gm x 10 Pkts</v>
       </c>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A229" s="2" t="s">
         <v>630</v>
       </c>
@@ -9264,7 +9263,7 @@
         <v>TORTILLA WRAPS PLAIN 8"570 gm</v>
       </c>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A230" s="2" t="s">
         <v>633</v>
       </c>
@@ -9294,7 +9293,7 @@
         <v>TORTILLA WRAPS PLAIN 10.5 INCHES875 gm x 10 Pkts</v>
       </c>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
         <v>635</v>
       </c>
@@ -9324,7 +9323,7 @@
         <v>TORTILLA WRAPS HOT  N  SPICY 8"570 gm</v>
       </c>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
         <v>637</v>
       </c>
@@ -9354,7 +9353,7 @@
         <v>GREEN PEAS400 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" s="2" t="s">
         <v>639</v>
       </c>
@@ -9384,7 +9383,7 @@
         <v>GREEN PEAS 900900 gm x 10 Pkts</v>
       </c>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
         <v>641</v>
       </c>
@@ -9414,7 +9413,7 @@
         <v>Green Peas with Carrots400 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
         <v>643</v>
       </c>
@@ -9444,7 +9443,7 @@
         <v>Green Peas with Carrots 900900 gm x 10 Pkts</v>
       </c>
     </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A236" s="2" t="s">
         <v>645</v>
       </c>
@@ -9474,7 +9473,7 @@
         <v>MIXED VEGETABLES 400400 gm x 20 Pkts</v>
       </c>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
         <v>647</v>
       </c>
@@ -9504,7 +9503,7 @@
         <v>MIXED VEGETABLES 900900 gm x 10 Pkts</v>
       </c>
     </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
         <v>649</v>
       </c>

</xml_diff>